<commit_message>
feat(sheets): clean template without dummy data and update links to active Google Sheet
</commit_message>
<xml_diff>
--- a/TagX_Website_Database_Template.xlsx
+++ b/TagX_Website_Database_Template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +31,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Plus Jakarta Sans"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -83,16 +79,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -462,21 +452,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="111" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
@@ -520,147 +510,6 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Founder Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 22:45</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>TX-1001</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Sundar Pitchai (Apex FinTech)</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>sundar@apexfin.io</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>3D WebGL Web Experiences</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Need a high-performance 3D interactive landing page with WebGL laptop model for our Series-A SaaS launch.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>,500 - ,000</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>High priority - send deck</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 21:15</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>TX-1002</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Vikramaditya (Nova Labs)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>vikram@novalabs.tech</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Custom Software Development</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Scalable Node.js / Python API backend with real-time telemetry streaming and automated PDF/Excel reporting.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>,000 - ,500</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>In Review</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Schedule Google Meet demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 19:30</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>TX-1003</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Meenakshi (HealthGenix)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>meena@healthgenix.org</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Freelance Engineering</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Next.js 15 web application with secure patient portal, HIPAA compliance, and responsive mobile UI.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>₹1,50,000 - ₹3,00,000</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Contacted</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Awaiting requirement doc</t>
         </is>
       </c>
     </row>
@@ -675,157 +524,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Registration Timestamp</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Developer / User Email</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Access Tier</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Invitation Status</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Platform / Source</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Notes / Feedback</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 22:50</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>kavitha.dev@gmail.com</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>VIP Early Access 🚀</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Pending Launch</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Website Hero Section</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Requested Early Beta invite</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 21:40</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>rahul.ai@stanford.edu</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>VIP Early Access 🚀</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Pending Launch</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Products Bento Card</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Wants API integration access</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 18:20</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>alex.turner@cloudtech.co</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>VIP Early Access 🚀</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Pending Launch</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Website Freelance Footer</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Interested in in-house tools</t>
         </is>
       </c>
     </row>

</xml_diff>